<commit_message>
Add updated project elements
</commit_message>
<xml_diff>
--- a/data/workbooks/2014.xlsx
+++ b/data/workbooks/2014.xlsx
@@ -3,23 +3,23 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424AD0CD-1011-4293-814E-ECD461779792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93653976-B341-4E70-B8AC-73DAC6EBFFA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Январь 2014" sheetId="16" r:id="rId1"/>
-    <sheet name="Февраль 2014" sheetId="17" r:id="rId2"/>
-    <sheet name="Март 2014" sheetId="19" r:id="rId3"/>
-    <sheet name="Апрель 2014" sheetId="20" r:id="rId4"/>
-    <sheet name="Май 2014" sheetId="21" r:id="rId5"/>
-    <sheet name="Июнь 2014" sheetId="22" r:id="rId6"/>
-    <sheet name="Июль 2014" sheetId="23" r:id="rId7"/>
-    <sheet name="Август 2014" sheetId="24" r:id="rId8"/>
-    <sheet name="Сентябрь 2014" sheetId="25" r:id="rId9"/>
-    <sheet name="Октябрь 2014" sheetId="26" r:id="rId10"/>
-    <sheet name="Ноябрь 2014" sheetId="27" r:id="rId11"/>
-    <sheet name="Декабрь 2014" sheetId="28" r:id="rId12"/>
+    <sheet name="Січень 2014" sheetId="16" r:id="rId1"/>
+    <sheet name="Лютий 2014" sheetId="17" r:id="rId2"/>
+    <sheet name="Березень 2014" sheetId="19" r:id="rId3"/>
+    <sheet name="Квітень 2014" sheetId="20" r:id="rId4"/>
+    <sheet name="Травень 2014" sheetId="21" r:id="rId5"/>
+    <sheet name="Червень 2014" sheetId="22" r:id="rId6"/>
+    <sheet name="Липень 2014" sheetId="23" r:id="rId7"/>
+    <sheet name="Серпень 2014" sheetId="24" r:id="rId8"/>
+    <sheet name="Вересень 2014" sheetId="25" r:id="rId9"/>
+    <sheet name="Жовтень 2014" sheetId="26" r:id="rId10"/>
+    <sheet name="Листопад 2014" sheetId="27" r:id="rId11"/>
+    <sheet name="Грудень 2014" sheetId="28" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,39 +37,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="31">
-  <si>
-    <t>Доходы</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="33">
   <si>
     <t>Зарплата</t>
-  </si>
-  <si>
-    <t>Расходы</t>
-  </si>
-  <si>
-    <t>Потребности</t>
-  </si>
-  <si>
-    <t>Развлечения</t>
   </si>
   <si>
     <t>Квартира</t>
   </si>
   <si>
-    <t>Проезд</t>
-  </si>
-  <si>
-    <t>Долги</t>
-  </si>
-  <si>
-    <t>Другое</t>
-  </si>
-  <si>
     <t>Алкоголь</t>
-  </si>
-  <si>
-    <t>Всего</t>
   </si>
   <si>
     <t>вс</t>
@@ -93,43 +69,73 @@
     <t>пн</t>
   </si>
   <si>
-    <t>Всего за месяц</t>
-  </si>
-  <si>
     <t>%</t>
-  </si>
-  <si>
-    <t>Прибыль</t>
-  </si>
-  <si>
-    <t>Здоровье</t>
-  </si>
-  <si>
-    <t>Хоз.Товары</t>
-  </si>
-  <si>
-    <t>В среднем</t>
-  </si>
-  <si>
-    <t>Питание</t>
-  </si>
-  <si>
-    <t>Другие доходы</t>
-  </si>
-  <si>
-    <t>Баланс на нач. мес.</t>
-  </si>
-  <si>
-    <t>Баланс на кон. мес.</t>
-  </si>
-  <si>
-    <t>Мероприятия</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>Закуски</t>
+    <t>Доходи</t>
+  </si>
+  <si>
+    <t>Інші доходи</t>
+  </si>
+  <si>
+    <t>Витрати</t>
+  </si>
+  <si>
+    <t>Потреби</t>
+  </si>
+  <si>
+    <t>Харчування</t>
+  </si>
+  <si>
+    <t>Проїзд</t>
+  </si>
+  <si>
+    <t>Здоров'я</t>
+  </si>
+  <si>
+    <t>Госп.Товари</t>
+  </si>
+  <si>
+    <t>Борги</t>
+  </si>
+  <si>
+    <t>Інші витрати</t>
+  </si>
+  <si>
+    <t>Необов'язкове</t>
+  </si>
+  <si>
+    <t>Заходи</t>
+  </si>
+  <si>
+    <t>Розваги</t>
+  </si>
+  <si>
+    <t>Всього</t>
+  </si>
+  <si>
+    <t>Баланс на поч. міс.</t>
+  </si>
+  <si>
+    <t>Прибуток</t>
+  </si>
+  <si>
+    <t>Баланс на кін. міс.</t>
+  </si>
+  <si>
+    <t>нд</t>
+  </si>
+  <si>
+    <t>В середньому</t>
+  </si>
+  <si>
+    <t>Всього за місяць</t>
+  </si>
+  <si>
+    <t>Смаколики</t>
   </si>
 </sst>
 </file>
@@ -702,14 +708,14 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1137,7 +1143,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.5703125" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -1148,106 +1154,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="I1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="O1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="P1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="R1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="T1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="V1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="W1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Y1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="Z1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AA1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AC1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AD1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AE1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AF1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AG1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AH1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1353,11 +1359,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -1410,7 +1416,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -1458,13 +1464,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2"/>
@@ -1542,7 +1548,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4">
@@ -1642,7 +1648,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -1698,7 +1704,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -1758,7 +1764,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -1814,7 +1820,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -1870,7 +1876,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2"/>
@@ -1927,10 +1933,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6">
         <v>19</v>
@@ -1994,7 +2000,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -2050,7 +2056,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -2102,7 +2108,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51">
@@ -2165,7 +2171,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -2272,7 +2278,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -2319,7 +2325,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -2400,7 +2406,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.7109375" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -2411,106 +2417,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="I1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="O1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="P1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="R1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="T1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="V1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="W1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Y1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="Z1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AA1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AC1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AD1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AE1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AF1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AG1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AH1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2616,11 +2622,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -2673,7 +2679,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -2719,13 +2725,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21">
         <v>86</v>
@@ -2815,7 +2821,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4">
         <v>12</v>
@@ -2921,7 +2927,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25">
         <v>11</v>
@@ -2977,7 +2983,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38">
         <v>2</v>
@@ -3051,7 +3057,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -3105,7 +3111,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -3155,7 +3161,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2"/>
@@ -3232,10 +3238,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -3295,7 +3301,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -3351,7 +3357,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -3423,7 +3429,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -3474,7 +3480,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -3581,7 +3587,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -3628,7 +3634,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -3672,7 +3678,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -3714,7 +3720,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.28515625" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -3725,104 +3731,104 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E1" s="37" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="M1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="O1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="S1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="T1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="V1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="Y1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Z1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AA1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AC1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AD1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AE1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AG1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AH1" s="56"/>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3928,11 +3934,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -3983,7 +3989,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -4027,13 +4033,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2"/>
@@ -4111,7 +4117,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4">
         <v>6</v>
@@ -4209,7 +4215,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -4259,7 +4265,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -4313,7 +4319,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -4367,7 +4373,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -4417,7 +4423,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21">
         <v>78</v>
@@ -4492,10 +4498,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6">
@@ -4551,7 +4557,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -4603,7 +4609,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6">
         <v>13</v>
@@ -4681,7 +4687,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -4736,7 +4742,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -4843,7 +4849,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -4890,7 +4896,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -4934,7 +4940,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -4976,7 +4982,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.85546875" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -4987,106 +4993,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="K1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="O1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Q1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="R1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="T1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="V1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="X1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="Y1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Z1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AA1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AC1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AD1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AE1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AF1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AG1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AH1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -5192,11 +5198,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -5251,7 +5257,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -5293,13 +5299,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21">
         <v>9</v>
@@ -5371,7 +5377,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4">
         <v>28</v>
@@ -5465,7 +5471,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -5515,7 +5521,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -5569,7 +5575,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -5621,7 +5627,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -5671,7 +5677,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2">
@@ -5730,10 +5736,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -5799,7 +5805,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -5851,7 +5857,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -5913,7 +5919,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -5968,7 +5974,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -6075,7 +6081,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -6122,7 +6128,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -6166,7 +6172,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -6208,7 +6214,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.42578125" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -6219,106 +6225,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="M1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="O1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="S1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="T1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="V1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="Y1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Z1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AA1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AC1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AD1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AE1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AG1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AH1" s="36" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6424,11 +6430,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -6481,7 +6487,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18">
         <v>20</v>
@@ -6529,13 +6535,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2">
@@ -6615,7 +6621,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4">
@@ -6711,7 +6717,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -6765,7 +6771,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -6823,7 +6829,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -6877,7 +6883,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -6929,7 +6935,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21">
         <v>27</v>
@@ -6984,10 +6990,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -7047,7 +7053,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -7099,7 +7105,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -7151,7 +7157,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51">
         <v>50</v>
@@ -7208,7 +7214,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -7315,7 +7321,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -7362,7 +7368,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -7443,7 +7449,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.28515625" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -7454,106 +7460,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="M1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="O1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="S1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="T1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="V1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="Y1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Z1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AA1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AC1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AD1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AE1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AG1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AH1" s="36" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -7659,11 +7665,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -7716,7 +7722,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18">
         <v>20</v>
@@ -7768,13 +7774,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2">
@@ -7858,7 +7864,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4">
@@ -7960,7 +7966,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -8012,7 +8018,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -8072,7 +8078,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -8126,7 +8132,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -8176,7 +8182,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2"/>
@@ -8237,10 +8243,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -8308,7 +8314,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -8360,7 +8366,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6">
         <v>100</v>
@@ -8414,7 +8420,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -8473,7 +8479,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -8580,7 +8586,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -8627,7 +8633,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -8708,7 +8714,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.42578125" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -8719,106 +8725,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="J1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="O1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="P1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="Q1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="S1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="T1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="V1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="W1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="X1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Y1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Z1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AA1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AC1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AD1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AE1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AG1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AH1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8924,11 +8930,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -8983,7 +8989,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -9035,13 +9041,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2">
@@ -9125,7 +9131,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4">
         <v>6</v>
@@ -9227,7 +9233,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -9279,7 +9285,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -9339,7 +9345,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -9391,7 +9397,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -9441,7 +9447,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21">
         <v>40</v>
@@ -9504,10 +9510,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -9575,7 +9581,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -9631,7 +9637,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -9685,7 +9691,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -9746,7 +9752,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -9853,7 +9859,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -9900,7 +9906,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -9944,7 +9950,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -9986,7 +9992,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.5703125" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -9997,106 +10003,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="H1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="N1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="O1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Q1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="T1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="U1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="V1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="X1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="Y1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="Z1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AA1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AB1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AC1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AD1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AE1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AG1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AH1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -10202,11 +10208,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -10259,7 +10265,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18">
         <v>10</v>
@@ -10315,13 +10321,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2"/>
@@ -10413,7 +10419,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -10505,7 +10511,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -10561,7 +10567,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -10623,7 +10629,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -10679,7 +10685,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -10729,7 +10735,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2"/>
@@ -10792,10 +10798,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6">
         <v>18</v>
@@ -10869,7 +10875,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28">
         <v>18</v>
@@ -10923,7 +10929,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -10975,7 +10981,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51">
         <v>50</v>
@@ -11026,7 +11032,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -11133,7 +11139,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -11180,7 +11186,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -11224,7 +11230,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -11266,7 +11272,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.140625" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -11277,104 +11283,104 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="E1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="K1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="L1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="N1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="O1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="R1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="S1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="T1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="U1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="V1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Y1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="Z1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AA1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AB1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AC1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AD1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AE1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AF1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AG1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AH1" s="36"/>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -11480,11 +11486,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -11539,7 +11545,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18">
         <v>30</v>
@@ -11587,13 +11593,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2">
@@ -11695,7 +11701,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4">
         <v>27</v>
@@ -11787,7 +11793,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -11837,7 +11843,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -11901,7 +11907,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -11957,7 +11963,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -12009,7 +12015,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2">
@@ -12070,10 +12076,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6">
@@ -12143,7 +12149,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -12201,7 +12207,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -12251,7 +12257,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -12304,7 +12310,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="71"/>
@@ -12408,7 +12414,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -12455,7 +12461,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -12499,7 +12505,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -12540,7 +12546,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.5703125" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -12551,106 +12557,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="J1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="M1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="O1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="P1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="Q1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="S1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="T1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="V1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="W1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="X1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Y1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Z1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AA1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AC1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AD1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AE1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AG1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AH1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -12756,11 +12762,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -12811,7 +12817,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -12857,13 +12863,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21">
         <v>7</v>
@@ -12963,7 +12969,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4">
         <v>30</v>
@@ -13033,7 +13039,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -13087,7 +13093,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -13149,7 +13155,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21">
         <v>500</v>
@@ -13203,7 +13209,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -13253,7 +13259,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2"/>
@@ -13316,10 +13322,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6">
         <v>150</v>
@@ -13405,7 +13411,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28">
         <v>22</v>
@@ -13465,7 +13471,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -13521,7 +13527,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51">
@@ -13582,7 +13588,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -13689,7 +13695,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -13736,7 +13742,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -13780,7 +13786,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -13822,7 +13828,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.28515625" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -13833,106 +13839,106 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="G1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="J1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="K1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="M1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="N1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="O1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="P1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="Q1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="R1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="T1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="U1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="V1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="W1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="Y1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="Z1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AA1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AB1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AC1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AD1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AE1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AG1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AH1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -14038,11 +14044,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -14097,7 +14103,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -14139,13 +14145,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21">
         <v>14</v>
@@ -14229,7 +14235,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4">
@@ -14301,7 +14307,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -14355,7 +14361,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39"/>
@@ -14415,7 +14421,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -14467,7 +14473,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -14517,7 +14523,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2"/>
@@ -14574,10 +14580,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -14639,7 +14645,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -14689,7 +14695,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -14739,7 +14745,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -14788,7 +14794,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -14895,7 +14901,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -14942,7 +14948,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -14986,7 +14992,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -15028,7 +15034,7 @@
     <col min="2" max="2" width="6.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.28515625" style="1" customWidth="1"/>
     <col min="4" max="34" width="5.7109375" style="1" customWidth="1"/>
-    <col min="35" max="35" width="8.85546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="11.28515625" style="1" customWidth="1"/>
     <col min="36" max="36" width="10.140625" style="1" customWidth="1"/>
     <col min="37" max="37" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="38" max="16384" width="9.140625" style="1"/>
@@ -15039,104 +15045,104 @@
       <c r="B1" s="82"/>
       <c r="C1" s="83"/>
       <c r="D1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="K1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="N1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="O1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="P1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Q1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="R1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="T1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="U1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="V1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="W1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="X1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="Y1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="Z1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AA1" s="37" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="AB1" s="36" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AC1" s="36" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AD1" s="36" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AE1" s="37" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="AF1" s="56" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="AG1" s="36" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AH1" s="37"/>
       <c r="AI1" s="86" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="AJ1" s="95" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="AK1" s="97" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -15242,11 +15248,11 @@
     </row>
     <row r="3" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="99" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B3" s="100"/>
       <c r="C3" s="58" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -15301,7 +15307,7 @@
       <c r="A4" s="101"/>
       <c r="B4" s="102"/>
       <c r="C4" s="59" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="18"/>
@@ -15343,13 +15349,13 @@
     </row>
     <row r="5" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="88" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D5" s="21"/>
       <c r="E5" s="2">
@@ -15437,7 +15443,7 @@
       <c r="A6" s="89"/>
       <c r="B6" s="91"/>
       <c r="C6" s="61" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -15529,7 +15535,7 @@
       <c r="A7" s="89"/>
       <c r="B7" s="91"/>
       <c r="C7" s="61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="4"/>
@@ -15581,7 +15587,7 @@
       <c r="A8" s="89"/>
       <c r="B8" s="91"/>
       <c r="C8" s="62" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D8" s="38"/>
       <c r="E8" s="39">
@@ -15649,7 +15655,7 @@
       <c r="A9" s="89"/>
       <c r="B9" s="91"/>
       <c r="C9" s="60" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="2"/>
@@ -15701,7 +15707,7 @@
       <c r="A10" s="89"/>
       <c r="B10" s="91"/>
       <c r="C10" s="61" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -15751,7 +15757,7 @@
       <c r="A11" s="89"/>
       <c r="B11" s="91"/>
       <c r="C11" s="61" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="2"/>
@@ -15810,10 +15816,10 @@
     <row r="12" spans="1:37" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="89"/>
       <c r="B12" s="92" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -15869,7 +15875,7 @@
       <c r="A13" s="89"/>
       <c r="B13" s="93"/>
       <c r="C13" s="63" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="28"/>
       <c r="E13" s="8"/>
@@ -15921,7 +15927,7 @@
       <c r="A14" s="89"/>
       <c r="B14" s="93"/>
       <c r="C14" s="57" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
@@ -15983,7 +15989,7 @@
       <c r="A15" s="89"/>
       <c r="B15" s="94"/>
       <c r="C15" s="63" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="51"/>
@@ -16032,7 +16038,7 @@
     <row r="16" spans="1:37" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="90"/>
       <c r="B16" s="79" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="C16" s="80"/>
       <c r="D16" s="79">
@@ -16139,7 +16145,7 @@
     </row>
     <row r="18" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="108" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B18" s="108"/>
       <c r="C18" s="109"/>
@@ -16186,7 +16192,7 @@
     </row>
     <row r="19" spans="1:37" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="107" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="108"/>
       <c r="C19" s="109"/>
@@ -16230,7 +16236,7 @@
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.3">
       <c r="S24" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>